<commit_message>
Rebrand header and add Reefer (RF container) table
- Header: ship emoji replaces the plain dot, title is now "BSA
  Utilization Report", subtitle lists the tracked destination ports.
- New Reefer table (Excel sheet + dashboard section) computed from the
  booking file's RFCNT column (e.g. "45REx2" -> 2 reefer boxes),
  aggregated per sailing and destination port group, matching the
  layout of Report.xlsx's original Reefer sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Daily_Booking_Status_Report.xlsx
+++ b/Daily_Booking_Status_Report.xlsx
@@ -13,7 +13,8 @@
     <sheet name="POD - CNSHA" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="POD - IDJKT" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="POD - TOTAL,KR,JP,RU" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Alerts (OVER, FULL)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Reefer" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Alerts (OVER, FULL)" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Weekly Summary'!$A$1:$K$1</definedName>
@@ -22,6 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'POD - CNSHA'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'POD - IDJKT'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'POD - TOTAL,KR,JP,RU'!$A$1:$T$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reefer'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +47,9 @@
     <font>
       <b val="1"/>
       <color rgb="000000FF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -112,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +142,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -9584,6 +9590,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vessel / Voyage</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Reefer Qty</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>VNSGN Reefer Qty</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>JP Reefer Qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DONGJIN CONFIDENT (DJCF 0151N)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PEGASUS PROTO (PGPO 2611N)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr"/>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr"/>
+      <c r="D4" s="12" t="inlineStr"/>
+      <c r="E4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9600,52 +9748,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>SVC</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Vessel / Voyage</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>BSA</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>ALLO</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>LIFTING</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>TEU Note</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Excess TEU</t>
         </is>

</xml_diff>

<commit_message>
Fix reefer detection: use RF column, not sparsely-filled RFCNT
RFCNT ("45REx2") turned out to be filled in on only 2 of the 148 actual
reefer booking lines, so the Reefer table was massively undercounting.
The real signal is the RF column (e.g. "RF// MIN:-18.0 MAX:-18.0
[COVER:CLOSE]") being non-blank; that line's own container count
(C20+C40+C45) is the reefer quantity, confirmed against the 2 rows where
RFCNT's number happened to agree. Now picks up all 148 reefer lines
across 29 sailings (201 total reefer boxes) instead of just 2 lines.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Daily_Booking_Status_Report.xlsx
+++ b/Daily_Booking_Status_Report.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'POD - CNSHA'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'POD - IDJKT'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'POD - TOTAL,KR,JP,RU'!$A$1:$T$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reefer'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reefer'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9590,7 +9590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9600,6 +9600,12 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9635,7 +9641,37 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>HKHKG Reefer Qty</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>CNXMN Reefer Qty</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>CNSHK Reefer Qty</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>KR Reefer Qty</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>JP Reefer Qty</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RU Reefer Qty</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>IDJKT Reefer Qty</t>
         </is>
       </c>
     </row>
@@ -9647,12 +9683,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NTX</t>
+          <t>ANX</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DONGJIN CONFIDENT (DJCF 0151N)</t>
+          <t>INCHEON VOYAGER (ICVY 2607S)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -9661,13 +9697,31 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -9678,50 +9732,1409 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>ANX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>STARSHIP JUPITER (NSSJ 2607S)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ANX</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KMTC SURABAYA (KMSU 2607S)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA (SWMM 2609N)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>23</v>
+      </c>
+      <c r="F5" t="n">
+        <v>16</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KHS1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SAWASDEE INCHEON (SWIC 2610N)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KMTC ULSAN (KUS 2615N)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KTS1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA (KJT 2610N)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KTS1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CA MANILA (CMA 2614N)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>NTX</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DONGJIN CONFIDENT (DJCF 0151N)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SAWASDEE BALTIC (SWBT 2615N)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>11</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>PEGASUS PROTO (PGPO 2611N)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="K12" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Week 39</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>VTS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SKY ORION (SKOR 2611N)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>9</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA (SWSP 2609N)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CHT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KMTC GWANGYANG (KMGY 2610N)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CHT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB (SWDN 2610N)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>KHS1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK (KMBK 2611N)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>KST</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SAWASDEE ALTAIR (SWAL 2608N)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KTS1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC (SWAT 2610N)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Week 40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PCI2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SAWASDEE VEGA (SWVG 2612N)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Week 41</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNMAPPED (no SVC/schedule match)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SWCP (SWCP 2610N)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Week 41</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VTS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE (SWSR 2611N)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Week 41</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VTS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS (KMTP 2612N)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Week 42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA (SWMM 2610N)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>10</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Week 42</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DONGJIN CONFIDENT (DJCF 0152N)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Week 42</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NTX</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SAWASDEE BALTIC (SWBT 2616N)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>7</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Week 42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>VTS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SKY ORION (SKOR 2612N)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Week 43</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA (SWSP 2610N)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>10</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Week 43</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CHT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KMTC GWANGYANG (KMGY 2611N)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Week 44</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>KTS1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC (SWAT 2611N)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr"/>
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr"/>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>1</v>
+      <c r="C31" s="12" t="inlineStr"/>
+      <c r="D31" s="12" t="inlineStr"/>
+      <c r="E31" s="12" t="n">
+        <v>201</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="J31" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="K31" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="L31" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="M31" s="12" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Show N/A instead of "UNMAPPED (no SVC/schedule match)"
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Daily_Booking_Status_Report.xlsx
+++ b/Daily_Booking_Status_Report.xlsx
@@ -1524,7 +1524,7 @@
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>UNMAPPED (no SVC/schedule match)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5468,7 +5468,7 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>UNMAPPED (no SVC/schedule match)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -7619,7 +7619,7 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>UNMAPPED (no SVC/schedule match)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>UNMAPPED (no SVC/schedule match)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">

</xml_diff>

<commit_message>
Switch status colors to red=OK, blue=OVER, green=100%
Per the user's explicit (confirmed) instruction, the status palette is
now red for within-quota, blue for over-quota, and green for exactly
100%, applied across the dashboard (KPI cards, pills, percent text,
tooltip header, icons) and the Excel fills/emoji. The slot-share
"USE 60%" label stays blue independent of status.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Daily_Booking_Status_Report.xlsx
+++ b/Daily_Booking_Status_Report.xlsx
@@ -66,12 +66,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,7 +101,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -620,7 +620,7 @@
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K2" s="3" t="n">
@@ -660,7 +660,7 @@
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K3" s="3" t="n">
@@ -700,7 +700,7 @@
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K4" s="3" t="n">
@@ -740,7 +740,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K5" s="4" t="n">
@@ -780,7 +780,7 @@
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K6" s="3" t="n">
@@ -820,7 +820,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K7" s="4" t="n">
@@ -860,7 +860,7 @@
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K8" s="3" t="n">
@@ -900,7 +900,7 @@
       <c r="I9" s="3" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K9" s="3" t="n">
@@ -940,7 +940,7 @@
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K10" s="4" t="n">
@@ -980,7 +980,7 @@
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K11" s="3" t="n">
@@ -1020,7 +1020,7 @@
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K12" s="4" t="n">
@@ -1060,7 +1060,7 @@
       <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K13" s="3" t="n">
@@ -1100,7 +1100,7 @@
       <c r="I14" s="3" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K14" s="3" t="n">
@@ -1145,7 +1145,7 @@
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K15" s="4" t="n">
@@ -1185,7 +1185,7 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K16" s="4" t="n">
@@ -1225,7 +1225,7 @@
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K17" s="4" t="n">
@@ -1265,7 +1265,7 @@
       <c r="I18" s="3" t="inlineStr"/>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K18" s="3" t="n">
@@ -1305,7 +1305,7 @@
       <c r="I19" s="3" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K19" s="3" t="n">
@@ -1345,7 +1345,7 @@
       <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="K20" s="3" t="n">
@@ -1385,7 +1385,7 @@
       <c r="I21" s="4" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K21" s="4" t="n">
@@ -1430,7 +1430,7 @@
       <c r="I22" s="4" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K22" s="4" t="n">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K23" s="4" t="n">
@@ -1514,7 +1514,7 @@
       <c r="I24" s="4" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K24" s="4" t="n">
@@ -1598,7 +1598,7 @@
       <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K26" s="4" t="n">
@@ -1638,7 +1638,7 @@
       <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K27" s="4" t="n">
@@ -1683,7 +1683,7 @@
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K28" s="4" t="n">
@@ -1723,7 +1723,7 @@
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K29" s="4" t="n">
@@ -1763,7 +1763,7 @@
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K30" s="4" t="n">
@@ -1803,7 +1803,7 @@
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K31" s="4" t="n">
@@ -1843,7 +1843,7 @@
       <c r="I32" s="4" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K32" s="4" t="n">
@@ -1883,7 +1883,7 @@
       <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K33" s="4" t="n">
@@ -1923,7 +1923,7 @@
       <c r="I34" s="4" t="inlineStr"/>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K34" s="4" t="n">
@@ -1963,7 +1963,7 @@
       <c r="I35" s="4" t="inlineStr"/>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K35" s="4" t="n">
@@ -2003,7 +2003,7 @@
       <c r="I36" s="4" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K36" s="4" t="n">
@@ -2043,7 +2043,7 @@
       <c r="I37" s="4" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K37" s="4" t="n">
@@ -2088,7 +2088,7 @@
       <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K38" s="4" t="n">
@@ -2128,7 +2128,7 @@
       <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K39" s="4" t="n">
@@ -2168,7 +2168,7 @@
       <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K40" s="4" t="n">
@@ -2208,7 +2208,7 @@
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K41" s="4" t="n">
@@ -2248,7 +2248,7 @@
       <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K42" s="4" t="n">
@@ -2288,7 +2288,7 @@
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K43" s="4" t="n">
@@ -2328,7 +2328,7 @@
       <c r="I44" s="4" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K44" s="4" t="n">
@@ -2368,7 +2368,7 @@
       <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K45" s="4" t="n">
@@ -2408,7 +2408,7 @@
       <c r="I46" s="4" t="inlineStr"/>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K46" s="4" t="n">
@@ -2453,7 +2453,7 @@
       <c r="I47" s="4" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K47" s="4" t="n">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K48" s="4" t="n">
@@ -2537,7 +2537,7 @@
       <c r="I49" s="4" t="inlineStr"/>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K49" s="4" t="n">
@@ -2577,7 +2577,7 @@
       <c r="I50" s="4" t="inlineStr"/>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K50" s="4" t="n">
@@ -2617,7 +2617,7 @@
       <c r="I51" s="4" t="inlineStr"/>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K51" s="4" t="n">
@@ -2657,7 +2657,7 @@
       <c r="I52" s="4" t="inlineStr"/>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>🟢 OK</t>
+          <t>🔴 OK</t>
         </is>
       </c>
       <c r="K52" s="4" t="n">
@@ -11245,7 +11245,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J2" s="3" t="n">
@@ -11285,7 +11285,7 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J3" s="3" t="n">
@@ -11325,7 +11325,7 @@
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J4" s="3" t="n">
@@ -11365,7 +11365,7 @@
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J5" s="3" t="n">
@@ -11405,7 +11405,7 @@
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J6" s="3" t="n">
@@ -11445,7 +11445,7 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J7" s="3" t="n">
@@ -11485,7 +11485,7 @@
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J8" s="3" t="n">
@@ -11525,7 +11525,7 @@
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J9" s="3" t="n">
@@ -11565,7 +11565,7 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J10" s="3" t="n">
@@ -11605,7 +11605,7 @@
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J11" s="3" t="n">
@@ -11645,7 +11645,7 @@
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J12" s="3" t="n">
@@ -11685,7 +11685,7 @@
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>🔴 OVER</t>
+          <t>🔵 OVER</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">

</xml_diff>

<commit_message>
Rename the red status label from "OK" to "Dangerous"
Display-only rename (KPI card, status filter, pills, Excel status text);
internal status keys and the under-quota logic are unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Daily_Booking_Status_Report.xlsx
+++ b/Daily_Booking_Status_Report.xlsx
@@ -740,7 +740,7 @@
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K5" s="4" t="n">
@@ -820,7 +820,7 @@
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K7" s="4" t="n">
@@ -940,7 +940,7 @@
       <c r="I10" s="4" t="inlineStr"/>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K10" s="4" t="n">
@@ -1020,7 +1020,7 @@
       <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K12" s="4" t="n">
@@ -1145,7 +1145,7 @@
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K15" s="4" t="n">
@@ -1185,7 +1185,7 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K16" s="4" t="n">
@@ -1225,7 +1225,7 @@
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K17" s="4" t="n">
@@ -1385,7 +1385,7 @@
       <c r="I21" s="4" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K21" s="4" t="n">
@@ -1430,7 +1430,7 @@
       <c r="I22" s="4" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K22" s="4" t="n">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K23" s="4" t="n">
@@ -1514,7 +1514,7 @@
       <c r="I24" s="4" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K24" s="4" t="n">
@@ -1598,7 +1598,7 @@
       <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K26" s="4" t="n">
@@ -1638,7 +1638,7 @@
       <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K27" s="4" t="n">
@@ -1683,7 +1683,7 @@
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K28" s="4" t="n">
@@ -1723,7 +1723,7 @@
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K29" s="4" t="n">
@@ -1763,7 +1763,7 @@
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K30" s="4" t="n">
@@ -1803,7 +1803,7 @@
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K31" s="4" t="n">
@@ -1843,7 +1843,7 @@
       <c r="I32" s="4" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K32" s="4" t="n">
@@ -1883,7 +1883,7 @@
       <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K33" s="4" t="n">
@@ -1923,7 +1923,7 @@
       <c r="I34" s="4" t="inlineStr"/>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K34" s="4" t="n">
@@ -1963,7 +1963,7 @@
       <c r="I35" s="4" t="inlineStr"/>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K35" s="4" t="n">
@@ -2003,7 +2003,7 @@
       <c r="I36" s="4" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K36" s="4" t="n">
@@ -2043,7 +2043,7 @@
       <c r="I37" s="4" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K37" s="4" t="n">
@@ -2088,7 +2088,7 @@
       <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K38" s="4" t="n">
@@ -2128,7 +2128,7 @@
       <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K39" s="4" t="n">
@@ -2168,7 +2168,7 @@
       <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K40" s="4" t="n">
@@ -2208,7 +2208,7 @@
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K41" s="4" t="n">
@@ -2248,7 +2248,7 @@
       <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K42" s="4" t="n">
@@ -2288,7 +2288,7 @@
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K43" s="4" t="n">
@@ -2328,7 +2328,7 @@
       <c r="I44" s="4" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K44" s="4" t="n">
@@ -2368,7 +2368,7 @@
       <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K45" s="4" t="n">
@@ -2408,7 +2408,7 @@
       <c r="I46" s="4" t="inlineStr"/>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K46" s="4" t="n">
@@ -2453,7 +2453,7 @@
       <c r="I47" s="4" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K47" s="4" t="n">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K48" s="4" t="n">
@@ -2537,7 +2537,7 @@
       <c r="I49" s="4" t="inlineStr"/>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K49" s="4" t="n">
@@ -2577,7 +2577,7 @@
       <c r="I50" s="4" t="inlineStr"/>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K50" s="4" t="n">
@@ -2617,7 +2617,7 @@
       <c r="I51" s="4" t="inlineStr"/>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K51" s="4" t="n">
@@ -2657,7 +2657,7 @@
       <c r="I52" s="4" t="inlineStr"/>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>🔴 OK</t>
+          <t>🔴 Dangerous</t>
         </is>
       </c>
       <c r="K52" s="4" t="n">

</xml_diff>